<commit_message>
Complete Sprint 6 API and analytics
</commit_message>
<xml_diff>
--- a/exports/peer_comparison.xlsx
+++ b/exports/peer_comparison.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -556,7 +556,7 @@
         <v>22.17</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>50</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>24.2</v>
@@ -568,13 +568,13 @@
         <v>0.02321972845663619</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>87.5</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>890</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>37.5</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="L2" s="2" t="n">
         <v/>
@@ -590,31 +590,31 @@
         <v>95</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>81.25</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>26.61</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>81.25</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>17.18</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>81.25</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0.06601754022512257</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>56.25</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>6486</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>81.25</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="L3" s="2" t="n">
         <v/>
@@ -623,38 +623,39 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Bajaj Auto Ltd</t>
+          <t xml:space="preserve">Hero MotoCorp Ltd
+</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>81.25</v>
+        <v>85</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>71.42857142857143</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>26.61</v>
+        <v>21.14</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>81.25</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>17.18</v>
+        <v>9.9</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>81.25</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.06601754022512257</v>
+        <v>0.03423922255494661</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>56.25</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>6486</v>
+        <v>3095</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>81.25</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="L4" s="2" t="n">
         <v/>
@@ -663,39 +664,38 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hero MotoCorp Ltd
-</t>
+          <t>Maruti Suzuki India Ltd</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>62.5</v>
+        <v>50</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>21.14</v>
+        <v>15.75</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>37.5</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>9.9</v>
+        <v>9.51</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>62.5</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.03423922255494661</v>
+        <v>0.001389602503619973</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>3095</v>
+        <v>4936</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>50</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="L5" s="2" t="n">
         <v/>
@@ -704,38 +704,38 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Maruti Suzuki India Ltd</t>
+          <t>Tata Motors Ltd</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
         <v>80</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>43.75</v>
+        <v>50</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>15.75</v>
+        <v>37.46</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>12.5</v>
+        <v>100</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>9.51</v>
+        <v>7.26</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>50</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.001389602503619973</v>
+        <v>1.263124425916767</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>100</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>4936</v>
+        <v>45133</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>62.5</v>
+        <v>100</v>
       </c>
       <c r="L6" s="2" t="n">
         <v/>
@@ -744,38 +744,39 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Tata Motors Ltd</t>
+          <t xml:space="preserve">Mahindra &amp; Mahindra Ltd
+</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>43.75</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>37.46</v>
+        <v>18.54</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>100</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>7.26</v>
+        <v>8.82</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>25</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.263124425916767</v>
+        <v>1.641441305333132</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>37.5</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>45133</v>
+        <v>-11245</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>100</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="L7" s="2" t="n">
         <v/>
@@ -784,122 +785,81 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mahindra &amp; Mahindra Ltd
-</t>
+          <t>TVS Motor Company Ltd</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>25</v>
+        <v>40</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>14.28571428571428</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>18.54</v>
+        <v>26.22</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>25</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>8.82</v>
+        <v>4.54</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>37.5</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1.641441305333132</v>
+        <v>3.833431603773585</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>25</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>-11245</v>
+        <v>-2254</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>12.5</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="L8" s="2" t="n">
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>TVS Motor Company Ltd</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>26.22</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>4.54</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>3.833431603773585</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>-2254</v>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="L9" s="2" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>MEDIAN</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>82.5</v>
-      </c>
-      <c r="C11" t="n">
-        <v>53.12</v>
-      </c>
-      <c r="D11" t="n">
-        <v>24.2</v>
-      </c>
-      <c r="E11" t="n">
-        <v>56.25</v>
-      </c>
-      <c r="F11" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="G11" t="n">
-        <v>56.25</v>
-      </c>
-      <c r="H11" t="n">
+      <c r="B10" t="n">
+        <v>80</v>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="n">
+        <v>22.17</v>
+      </c>
+      <c r="E10" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="F10" t="n">
+        <v>9.51</v>
+      </c>
+      <c r="G10" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="H10" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="I11" t="n">
-        <v>56.25</v>
-      </c>
-      <c r="J11" t="n">
-        <v>4015.5</v>
-      </c>
-      <c r="K11" t="n">
-        <v>56.25</v>
-      </c>
-      <c r="L11" t="n">
+      <c r="I10" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="J10" t="n">
+        <v>3095</v>
+      </c>
+      <c r="K10" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="L10" t="n">
         <v/>
       </c>
     </row>
@@ -914,7 +874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1009,19 +969,19 @@
         <v>16.72</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>28.57142857142857</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>13.94</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>85.71428571428571</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>14.86741992554242</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>14.28571428571428</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>13296</v>
@@ -1042,14 +1002,14 @@
       <c r="B3" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>85.71428571428571</v>
+      <c r="C3" s="4" t="n">
+        <v>66.66666666666666</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>15.76</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>14.28571428571428</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>15.94</v>
@@ -1061,13 +1021,13 @@
         <v>12.14371872728943</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>28.57142857142857</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>-7559</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>85.71428571428571</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="L3" s="2" t="n">
         <v/>
@@ -1083,234 +1043,74 @@
         <v>45</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>42.85714285714285</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>61.32</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>71.42857142857143</v>
+        <v>100</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>8.4</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>42.85714285714285</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>3.684256345007701</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>71.42857142857143</v>
+        <v>100</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>-29445</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>42.85714285714285</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="L4" s="2" t="n">
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Punjab National Bank</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>61.32</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>71.42857142857143</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>3.684256345007701</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>71.42857142857143</v>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>-29445</v>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="L5" s="2" t="n">
-        <v/>
-      </c>
-    </row>
+    <row r="5"/>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Punjab National Bank</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>61.32</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>71.42857142857143</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>3.684256345007701</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>71.42857142857143</v>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>-29445</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="L6" s="2" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Punjab National Bank</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>61.32</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>71.42857142857143</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>3.684256345007701</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>71.42857142857143</v>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>-29445</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Punjab National Bank</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>61.32</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>71.42857142857143</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>3.684256345007701</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>71.42857142857143</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>-29445</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>42.85714285714285</v>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>MEDIAN</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>45</v>
-      </c>
-      <c r="C10" t="n">
-        <v>42.86</v>
-      </c>
-      <c r="D10" t="n">
-        <v>61.32</v>
-      </c>
-      <c r="E10" t="n">
-        <v>71.43000000000001</v>
-      </c>
-      <c r="F10" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="G10" t="n">
-        <v>42.86</v>
-      </c>
-      <c r="H10" t="n">
-        <v>3.68</v>
-      </c>
-      <c r="I10" t="n">
-        <v>71.43000000000001</v>
-      </c>
-      <c r="J10" t="n">
-        <v>-29445</v>
-      </c>
-      <c r="K10" t="n">
-        <v>42.86</v>
-      </c>
-      <c r="L10" t="n">
+      <c r="B6" t="n">
+        <v>50</v>
+      </c>
+      <c r="C6" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16.72</v>
+      </c>
+      <c r="E6" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="F6" t="n">
+        <v>13.94</v>
+      </c>
+      <c r="G6" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="H6" t="n">
+        <v>12.14</v>
+      </c>
+      <c r="I6" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-7559</v>
+      </c>
+      <c r="K6" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="L6" t="n">
         <v/>
       </c>
     </row>
@@ -2282,7 +2082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2371,31 +2171,31 @@
         <v>95</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>91.66666666666666</v>
+        <v>90</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>29.79</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>83.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>17.08</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>83.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0.09486358890553362</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>66.66666666666666</v>
+        <v>60</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>20117</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>83.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="L2" s="2" t="n">
         <v/>
@@ -2411,31 +2211,31 @@
         <v>95</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>91.66666666666666</v>
+        <v>90</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>22.9</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>12.91</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0.1034568888000799</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>16.66666666666666</v>
+        <v>20</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1752</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>16.66666666666666</v>
+        <v>20</v>
       </c>
       <c r="L3" s="2" t="n">
         <v/>
@@ -2451,19 +2251,19 @@
         <v>90</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>58.33333333333334</v>
+        <v>50</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>23.01</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>66.66666666666666</v>
+        <v>60</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>14.29</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>66.66666666666666</v>
+        <v>60</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0.08435023365512796</v>
@@ -2475,7 +2275,7 @@
         <v>15840</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>66.66666666666666</v>
+        <v>60</v>
       </c>
       <c r="L4" s="2" t="n">
         <v/>
@@ -2491,7 +2291,7 @@
         <v>90</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>58.33333333333334</v>
+        <v>50</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>50.94</v>
@@ -2509,7 +2309,7 @@
         <v>0.0886406082507266</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>83.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>50429</v>
@@ -2530,115 +2330,75 @@
       <c r="B6" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="C6" s="4" t="n">
-        <v>25</v>
+      <c r="C6" s="5" t="n">
+        <v>20</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>8.99</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>4.61</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>0.09512917619708275</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>41.66666666666667</v>
+        <v>40</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>5058</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>41.66666666666667</v>
+        <v>40</v>
       </c>
       <c r="L6" s="2" t="n">
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Tech Mahindra Ltd</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
+    <row r="7"/>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>MEDIAN</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>90</v>
+      </c>
+      <c r="C8" t="n">
         <v>50</v>
       </c>
-      <c r="C7" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>4.61</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>0.09512917619708275</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>41.66666666666667</v>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>5058</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>41.66666666666667</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>MEDIAN</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>90</v>
-      </c>
-      <c r="C9" t="n">
-        <v>58.33</v>
-      </c>
-      <c r="D9" t="n">
-        <v>22.96</v>
-      </c>
-      <c r="E9" t="n">
-        <v>58.33</v>
-      </c>
-      <c r="F9" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="G9" t="n">
-        <v>58.33</v>
-      </c>
-      <c r="H9" t="n">
+      <c r="D8" t="n">
+        <v>23.01</v>
+      </c>
+      <c r="E8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F8" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="G8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H8" t="n">
         <v>0.09</v>
       </c>
-      <c r="I9" t="n">
-        <v>54.17</v>
-      </c>
-      <c r="J9" t="n">
-        <v>10449</v>
-      </c>
-      <c r="K9" t="n">
-        <v>54.17</v>
-      </c>
-      <c r="L9" t="n">
+      <c r="I8" t="n">
+        <v>60</v>
+      </c>
+      <c r="J8" t="n">
+        <v>15840</v>
+      </c>
+      <c r="K8" t="n">
+        <v>60</v>
+      </c>
+      <c r="L8" t="n">
         <v/>
       </c>
     </row>
@@ -3609,7 +3369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3710,7 +3470,7 @@
         <v>41.37</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>87.5</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0.8023177656738903</v>
@@ -3722,7 +3482,7 @@
         <v>17651</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>75</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="L2" s="2" t="n">
         <v/>
@@ -3738,31 +3498,31 @@
         <v>85</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>81.25</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>17.87</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>81.25</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>33.97</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>68.75</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>1.417345603929039</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>68.75</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>24176</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>93.75</v>
+        <v>100</v>
       </c>
       <c r="L3" s="2" t="n">
         <v/>
@@ -3771,38 +3531,39 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Power Grid Corporation of India Ltd</t>
+          <t xml:space="preserve">NHPC Ltd
+</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>81.25</v>
+        <v>80</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>71.42857142857143</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>17.87</v>
+        <v>10.41</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>81.25</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>33.97</v>
+        <v>41.82</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>68.75</v>
+        <v>100</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>1.417345603929039</v>
+        <v>0.8413260296625498</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>68.75</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>24176</v>
+        <v>970</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>93.75</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="L4" s="2" t="n">
         <v/>
@@ -3811,39 +3572,38 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NHPC Ltd
-</t>
+          <t>NTPC Ltd</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>62.5</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>10.41</v>
+        <v>13.27</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>25</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>41.82</v>
+        <v>11.95</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>100</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.8413260296625498</v>
+        <v>1.475521125007778</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>87.5</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>970</v>
+        <v>8644</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>37.5</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="L5" s="2" t="n">
         <v/>
@@ -3852,38 +3612,39 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NTPC Ltd</t>
+          <t xml:space="preserve">Tata Power Company Ltd
+</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>50</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>13.27</v>
+        <v>13.23</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>62.5</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>11.95</v>
+        <v>6.97</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>25</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1.475521125007778</v>
+        <v>1.659321300531586</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>50</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>8644</v>
+        <v>3569</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>62.5</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="L6" s="2" t="n">
         <v/>
@@ -3892,39 +3653,38 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tata Power Company Ltd
-</t>
+          <t>JSW Energy Ltd</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>37.5</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13.23</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>50</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>6.97</v>
+        <v>15.02</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>12.5</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.659321300531586</v>
+        <v>1.515600998463902</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>25</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>3569</v>
+        <v>-1963</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>50</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="L7" s="2" t="n">
         <v/>
@@ -3933,121 +3693,81 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>JSW Energy Ltd</t>
+          <t>Adani Green Energy Ltd</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>25</v>
+        <v>35</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>14.28571428571428</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>8.279999999999999</v>
+        <v>12.81</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>12.5</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="F8" s="2" t="n">
+        <v>13.67</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>42.85714285714285</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>6.595281675818589</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>14.28571428571428</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>-13347</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>14.28571428571428</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>MEDIAN</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>65</v>
+      </c>
+      <c r="C10" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="D10" t="n">
+        <v>13.23</v>
+      </c>
+      <c r="E10" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="F10" t="n">
         <v>15.02</v>
       </c>
-      <c r="G8" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>1.515600998463902</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>-1963</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Adani Green Energy Ltd</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>12.81</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>13.67</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>6.595281675818589</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>-13347</v>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="L9" s="2" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>MEDIAN</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>72.5</v>
-      </c>
-      <c r="C11" t="n">
-        <v>56.25</v>
-      </c>
-      <c r="D11" t="n">
-        <v>13.25</v>
-      </c>
-      <c r="E11" t="n">
-        <v>56.25</v>
-      </c>
-      <c r="F11" t="n">
-        <v>24.49</v>
-      </c>
-      <c r="G11" t="n">
-        <v>59.38</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="I11" t="n">
-        <v>59.38</v>
-      </c>
-      <c r="J11" t="n">
-        <v>6106.5</v>
-      </c>
-      <c r="K11" t="n">
-        <v>56.25</v>
-      </c>
-      <c r="L11" t="n">
+      <c r="G10" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I10" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="J10" t="n">
+        <v>3569</v>
+      </c>
+      <c r="K10" t="n">
+        <v>57.14</v>
+      </c>
+      <c r="L10" t="n">
         <v/>
       </c>
     </row>

</xml_diff>